<commit_message>
Brand spelling SDWorx everywhere, regenerated documents and screenshots
</commit_message>
<xml_diff>
--- a/public/files/Nike_DE_Onboarding_Checklist.xlsx
+++ b/public/files/Nike_DE_Onboarding_Checklist.xlsx
@@ -461,7 +461,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated for the SD Worx hackathon demo</t>
+          <t>Generated for the SDWorx hackathon demo</t>
         </is>
       </c>
     </row>
@@ -536,7 +536,7 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>SD Worx</t>
+          <t>SDWorx</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
@@ -554,7 +554,7 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>SD Worx</t>
+          <t>SDWorx</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">

</xml_diff>